<commit_message>
Fix: Products Bulk Upload discount issue fix
</commit_message>
<xml_diff>
--- a/test_data/product_test_data.xlsx
+++ b/test_data/product_test_data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="79">
   <si>
     <t>product_name</t>
   </si>
@@ -38,7 +38,7 @@
     <t>regular_price</t>
   </si>
   <si>
-    <t>discount_price</t>
+    <t>discount_percentage</t>
   </si>
   <si>
     <t>stock</t>
@@ -74,58 +74,91 @@
     <t>variant_regular_price</t>
   </si>
   <si>
-    <t>variant_discount_price</t>
+    <t>variant_discount_percentage</t>
   </si>
   <si>
     <t>variant_stock</t>
   </si>
   <si>
-    <t>X-Product 1</t>
+    <t>Adidas Stan Smith</t>
   </si>
   <si>
     <t>Men's Fashion</t>
   </si>
   <si>
-    <t>Polo</t>
+    <t>Test</t>
   </si>
   <si>
     <t>Adidas</t>
   </si>
   <si>
-    <t>Short desc</t>
-  </si>
-  <si>
-    <t>Long description</t>
+    <t>Iconic leather sneakers</t>
+  </si>
+  <si>
+    <t>A classic design that has stayed fresh for over 50 years.</t>
   </si>
   <si>
     <t>active</t>
   </si>
   <si>
-    <t>8GB/128GB</t>
-  </si>
-  <si>
-    <t>XP1-8-128</t>
-  </si>
-  <si>
-    <t>8/128</t>
+    <t>Size 9 - White</t>
+  </si>
+  <si>
+    <t>SS-9-WHT</t>
+  </si>
+  <si>
+    <t>White</t>
+  </si>
+  <si>
+    <t>Size 10 - White</t>
+  </si>
+  <si>
+    <t>SS-10-WHT</t>
+  </si>
+  <si>
+    <t>US Polo Signature Blazer</t>
+  </si>
+  <si>
+    <t>US Polo</t>
+  </si>
+  <si>
+    <t>Tailored fit formal blazer</t>
+  </si>
+  <si>
+    <t>Expertly crafted for a sharp, sophisticated look at any event.</t>
+  </si>
+  <si>
+    <t>Adidas Adicolor Hoodie</t>
+  </si>
+  <si>
+    <t>Cozy fleece pullover hoodie</t>
+  </si>
+  <si>
+    <t>Classic sporty style with the iconic trefoil logo.</t>
+  </si>
+  <si>
+    <t>Medium - Black</t>
+  </si>
+  <si>
+    <t>AH-M-BLK</t>
+  </si>
+  <si>
+    <t>M</t>
   </si>
   <si>
     <t>Black</t>
   </si>
   <si>
-    <t>12GB/256GB</t>
-  </si>
-  <si>
-    <t>XP1-12-256</t>
-  </si>
-  <si>
-    <t>12/256</t>
-  </si>
-  <si>
-    <t>Silver</t>
-  </si>
-  <si>
-    <t>X-Product 2</t>
+    <t>Large - Black</t>
+  </si>
+  <si>
+    <t>AH-L-BLK</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>US Polo Women V-Neck Tee</t>
   </si>
   <si>
     <t>Female Fashion</t>
@@ -134,73 +167,91 @@
     <t>Kamiz</t>
   </si>
   <si>
-    <t>X-Product 3</t>
+    <t>Soft cotton v-neck t-shirt</t>
+  </si>
+  <si>
+    <t>Essential everyday tee with a flattering feminine fit.</t>
+  </si>
+  <si>
+    <t>Adidas Stella McCartney Kamiz</t>
+  </si>
+  <si>
+    <t>Designer collaboration kamiz</t>
+  </si>
+  <si>
+    <t>High-fashion meets high-performance in this unique collection.</t>
+  </si>
+  <si>
+    <t>US Polo Aviator Sunglasses</t>
+  </si>
+  <si>
+    <t>Watch</t>
+  </si>
+  <si>
+    <t>Classic aviator style shades</t>
+  </si>
+  <si>
+    <t>Polarized lenses with a timeless gold-tone frame.</t>
+  </si>
+  <si>
+    <t>Adidas Ice Dive Perfume</t>
   </si>
   <si>
     <t>Perfume</t>
   </si>
   <si>
-    <t>US Polo</t>
-  </si>
-  <si>
-    <t>X-Product 4</t>
-  </si>
-  <si>
-    <t>Shirt</t>
-  </si>
-  <si>
-    <t>Variant 1</t>
-  </si>
-  <si>
-    <t>XP4-V1</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>White</t>
-  </si>
-  <si>
-    <t>Variant 2</t>
-  </si>
-  <si>
-    <t>XP4-V2</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>Blue</t>
-  </si>
-  <si>
-    <t>X-Product 5</t>
-  </si>
-  <si>
-    <t>Watch</t>
-  </si>
-  <si>
-    <t>X-Product 6</t>
+    <t>Ozonic cool aquatic scent</t>
+  </si>
+  <si>
+    <t>For the man who lives his life with thrills and intensity.</t>
+  </si>
+  <si>
+    <t>US Polo Sport Chronograph</t>
+  </si>
+  <si>
+    <t>Rugged outdoor sports watch</t>
+  </si>
+  <si>
+    <t>Multi-function dial with durable silicone strap.</t>
+  </si>
+  <si>
+    <t>Orange Strap</t>
+  </si>
+  <si>
+    <t>USC-ORG</t>
+  </si>
+  <si>
+    <t>One Size</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Black Strap</t>
+  </si>
+  <si>
+    <t>USC-BLK</t>
+  </si>
+  <si>
+    <t>Adidas Gym Bag</t>
+  </si>
+  <si>
+    <t>Durable training duffel bag</t>
+  </si>
+  <si>
+    <t>Multiple compartments to keep your gear organized.</t>
+  </si>
+  <si>
+    <t>US Polo Embroidered Panjabi</t>
   </si>
   <si>
     <t>Punjabi</t>
   </si>
   <si>
-    <t>X-Product 7</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>X-Product 8</t>
-  </si>
-  <si>
-    <t>inactive</t>
-  </si>
-  <si>
-    <t>X-Product 9</t>
-  </si>
-  <si>
-    <t>X-Product 10</t>
+    <t>Intricate hand-work panjabi</t>
+  </si>
+  <si>
+    <t>Perfect for festivals and traditional ceremonies.</t>
   </si>
 </sst>
 </file>
@@ -540,7 +591,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:21">
@@ -628,18 +679,21 @@
         <v>26</v>
       </c>
       <c r="G2">
-        <v>1000</v>
+        <v>9500</v>
       </c>
       <c r="H2">
-        <v>900</v>
+        <v>10</v>
       </c>
       <c r="I2">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
         <v>1</v>
       </c>
       <c r="N2" t="s">
@@ -651,17 +705,17 @@
       <c r="P2" t="s">
         <v>29</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2">
+        <v>9</v>
+      </c>
+      <c r="R2" t="s">
         <v>30</v>
       </c>
-      <c r="R2" t="s">
-        <v>31</v>
-      </c>
       <c r="S2">
-        <v>1000</v>
+        <v>9500</v>
       </c>
       <c r="T2">
-        <v>900</v>
+        <v>10</v>
       </c>
       <c r="U2">
         <v>20</v>
@@ -672,59 +726,62 @@
         <v>21</v>
       </c>
       <c r="O3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" t="s">
         <v>32</v>
       </c>
-      <c r="P3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>34</v>
+      <c r="Q3">
+        <v>10</v>
       </c>
       <c r="R3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="S3">
-        <v>1100</v>
+        <v>9500</v>
       </c>
       <c r="T3">
-        <v>1000</v>
+        <v>10</v>
       </c>
       <c r="U3">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:21">
       <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" t="s">
         <v>36</v>
       </c>
-      <c r="B4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" t="s">
-        <v>26</v>
-      </c>
       <c r="G4">
-        <v>2000</v>
+        <v>12000</v>
       </c>
       <c r="H4">
-        <v>1800</v>
+        <v>15</v>
       </c>
       <c r="I4">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
       <c r="N4" t="s">
@@ -733,75 +790,63 @@
     </row>
     <row r="5" spans="1:21">
       <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" t="s">
         <v>39</v>
       </c>
-      <c r="B5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" t="s">
-        <v>26</v>
-      </c>
       <c r="G5">
-        <v>3000</v>
+        <v>5500</v>
       </c>
       <c r="H5">
-        <v>2500</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="J5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
       <c r="N5" t="s">
         <v>27</v>
       </c>
+      <c r="O5" t="s">
+        <v>40</v>
+      </c>
+      <c r="P5" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>42</v>
+      </c>
+      <c r="R5" t="s">
+        <v>43</v>
+      </c>
+      <c r="S5">
+        <v>5500</v>
+      </c>
+      <c r="T5">
+        <v>5</v>
+      </c>
+      <c r="U5">
+        <v>30</v>
+      </c>
     </row>
     <row r="6" spans="1:21">
       <c r="A6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6">
-        <v>4000</v>
-      </c>
-      <c r="H6">
-        <v>3500</v>
-      </c>
-      <c r="I6">
-        <v>50</v>
-      </c>
-      <c r="N6" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="O6" t="s">
         <v>44</v>
@@ -813,42 +858,48 @@
         <v>46</v>
       </c>
       <c r="R6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="S6">
-        <v>4000</v>
+        <v>5500</v>
       </c>
       <c r="T6">
-        <v>3500</v>
+        <v>5</v>
       </c>
       <c r="U6">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:21">
       <c r="A7" t="s">
-        <v>42</v>
-      </c>
-      <c r="O7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" t="s">
         <v>48</v>
       </c>
-      <c r="P7" t="s">
+      <c r="C7" t="s">
         <v>49</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="s">
         <v>50</v>
       </c>
-      <c r="R7" t="s">
+      <c r="F7" t="s">
         <v>51</v>
       </c>
-      <c r="S7">
-        <v>4200</v>
-      </c>
-      <c r="T7">
-        <v>3700</v>
-      </c>
-      <c r="U7">
-        <v>25</v>
+      <c r="G7">
+        <v>1500</v>
+      </c>
+      <c r="I7">
+        <v>100</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="N7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:21">
@@ -856,30 +907,33 @@
         <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="G8">
-        <v>5000</v>
+        <v>8500</v>
       </c>
       <c r="H8">
-        <v>4500</v>
+        <v>20</v>
       </c>
       <c r="I8">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
         <v>1</v>
       </c>
       <c r="L8">
@@ -891,31 +945,31 @@
     </row>
     <row r="9" spans="1:21">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="F9" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="G9">
-        <v>6000</v>
+        <v>3500</v>
       </c>
       <c r="H9">
-        <v>5500</v>
+        <v>10</v>
       </c>
       <c r="I9">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K9">
         <v>1</v>
@@ -929,40 +983,28 @@
     </row>
     <row r="10" spans="1:21">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
         <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="G10">
-        <v>7000</v>
+        <v>1800</v>
       </c>
       <c r="H10">
-        <v>6500</v>
+        <v>5</v>
       </c>
       <c r="I10">
-        <v>50</v>
-      </c>
-      <c r="J10">
-        <v>1</v>
-      </c>
-      <c r="K10">
-        <v>1</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="N10" t="s">
         <v>27</v>
@@ -970,74 +1012,92 @@
     </row>
     <row r="11" spans="1:21">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>22</v>
+      </c>
+      <c r="C11" t="s">
+        <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="G11">
-        <v>8000</v>
+        <v>6500</v>
       </c>
       <c r="H11">
-        <v>7500</v>
+        <v>12</v>
       </c>
       <c r="I11">
-        <v>50</v>
+        <v>30</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
       </c>
       <c r="N11" t="s">
-        <v>59</v>
+        <v>27</v>
+      </c>
+      <c r="O11" t="s">
+        <v>66</v>
+      </c>
+      <c r="P11" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>68</v>
+      </c>
+      <c r="R11" t="s">
+        <v>69</v>
+      </c>
+      <c r="S11">
+        <v>6500</v>
+      </c>
+      <c r="T11">
+        <v>12</v>
+      </c>
+      <c r="U11">
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:21">
       <c r="A12" t="s">
-        <v>60</v>
-      </c>
-      <c r="B12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" t="s">
-        <v>25</v>
-      </c>
-      <c r="F12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G12">
-        <v>9000</v>
-      </c>
-      <c r="H12">
-        <v>8500</v>
-      </c>
-      <c r="I12">
-        <v>50</v>
-      </c>
-      <c r="J12">
-        <v>1</v>
-      </c>
-      <c r="M12">
-        <v>1</v>
-      </c>
-      <c r="N12" t="s">
-        <v>27</v>
+        <v>63</v>
+      </c>
+      <c r="O12" t="s">
+        <v>70</v>
+      </c>
+      <c r="P12" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>68</v>
+      </c>
+      <c r="R12" t="s">
+        <v>43</v>
+      </c>
+      <c r="S12">
+        <v>6500</v>
+      </c>
+      <c r="T12">
+        <v>12</v>
+      </c>
+      <c r="U12">
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:21">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
         <v>22</v>
@@ -1046,30 +1106,59 @@
         <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="E13" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="F13" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="G13">
-        <v>10000</v>
-      </c>
-      <c r="H13">
-        <v>9500</v>
+        <v>2800</v>
       </c>
       <c r="I13">
         <v>50</v>
       </c>
-      <c r="K13">
-        <v>1</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
       <c r="N13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14">
+        <v>4800</v>
+      </c>
+      <c r="H14">
+        <v>10</v>
+      </c>
+      <c r="I14">
+        <v>25</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>1</v>
+      </c>
+      <c r="N14" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>